<commit_message>
this version doesn't work properly
</commit_message>
<xml_diff>
--- a/autoprogram/vgpio/names mapper.xlsx
+++ b/autoprogram/vgpio/names mapper.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alessandro\projects\autoprogram\autoprogram\vgpio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A827BC-AB87-49C2-8DD9-9BDD0AB53044}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51D3AEAC-3F15-46E5-B143-84C9D163CFDC}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{4FBC6C86-D509-43E8-82AC-DBC3FF078B39}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
   <si>
     <t>Tool.End Stock Removal</t>
   </si>
@@ -231,6 +231,12 @@
   </si>
   <si>
     <t>Rollomatic.LibCurve.Data.Curves.ToolProfileCurve.sP2</t>
+  </si>
+  <si>
+    <t>Rollomatic.LibCurve.Data.Curves.ToolProfileCurve.sP1</t>
+  </si>
+  <si>
+    <t>Tool.Set 1.Common Data.sP1</t>
   </si>
 </sst>
 </file>
@@ -317,7 +323,47 @@
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -638,7 +684,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42B2EC4B-F913-4D75-A9F6-A45AE9F236E1}">
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="90.42578125" style="3" customWidth="1"/>
@@ -663,257 +709,271 @@
     </row>
     <row r="3" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B4" s="5" t="s">
         <v>65</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>50</v>
+        <v>15</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>49</v>
+        <v>17</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B34" s="3" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:B36">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:B37">
     <sortCondition ref="A1"/>
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A1:B3 A5:B1048576">
+    <cfRule type="duplicateValues" dxfId="4" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A4:B4">
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>

</xml_diff>